<commit_message>
Padroniza a nomenclatura de regime tributário da carteira
Regimes passam a ser: SIMPLES NACIONAL, LUCRO PRESUMIDO, LUCRO REAL,
LUCRO REAL TRIMESTRAL e ISENTA FEDERAL — no cadastro (lista) e no modelo de
importação. O cadastro preserva um valor legado que ainda não esteja na lista
(não sobrescreve ao editar). Nenhum cálculo depende do texto do regime.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FeuPtySB66b4dyfPk7TTLb
</commit_message>
<xml_diff>
--- a/public/modelo-importacao-clientes.xlsx
+++ b/public/modelo-importacao-clientes.xlsx
@@ -611,9 +611,7 @@
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="6" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
     <col min="11" max="12" width="24" customWidth="1"/>
@@ -905,10 +903,10 @@
       <formula1>"Matriz,Filial"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G10:G203">
-      <formula1>"Simples,Presumido,Real"</formula1>
+      <formula1>"SIMPLES NACIONAL,LUCRO PRESUMIDO,LUCRO REAL,LUCRO REAL TRIMESTRAL,ISENTA FEDERAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G4:G203">
-      <formula1>"Simples,Presumido,Real"</formula1>
+      <formula1>"SIMPLES NACIONAL,LUCRO PRESUMIDO,LUCRO REAL,LUCRO REAL TRIMESTRAL,ISENTA FEDERAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H10:H203">
       <formula1>"Consolidado,Individualizado"</formula1>

</xml_diff>

<commit_message>
Padroniza a nomenclatura de regime tributário (#70)
Regimes passam a ser: SIMPLES NACIONAL, LUCRO PRESUMIDO, LUCRO REAL,
LUCRO REAL TRIMESTRAL e ISENTA FEDERAL — no cadastro (lista) e no modelo de
importação. O cadastro preserva um valor legado que ainda não esteja na lista
(não sobrescreve ao editar). Nenhum cálculo depende do texto do regime.


Claude-Session: https://claude.ai/code/session_01FeuPtySB66b4dyfPk7TTLb

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelo-importacao-clientes.xlsx
+++ b/public/modelo-importacao-clientes.xlsx
@@ -611,9 +611,7 @@
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="6" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
     <col min="11" max="12" width="24" customWidth="1"/>
@@ -905,10 +903,10 @@
       <formula1>"Matriz,Filial"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G10:G203">
-      <formula1>"Simples,Presumido,Real"</formula1>
+      <formula1>"SIMPLES NACIONAL,LUCRO PRESUMIDO,LUCRO REAL,LUCRO REAL TRIMESTRAL,ISENTA FEDERAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G4:G203">
-      <formula1>"Simples,Presumido,Real"</formula1>
+      <formula1>"SIMPLES NACIONAL,LUCRO PRESUMIDO,LUCRO REAL,LUCRO REAL TRIMESTRAL,ISENTA FEDERAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H10:H203">
       <formula1>"Consolidado,Individualizado"</formula1>

</xml_diff>